<commit_message>
All dynamics equations from Quang's online documentation into initial tech report document
</commit_message>
<xml_diff>
--- a/tables/Equation Table.xlsx
+++ b/tables/Equation Table.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\davisbr\Documents\SalmonMSE-Tech-Report\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\davisbr\Documents\SalmonMSE-Tech-Report\tables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{392AD780-2325-4C86-BAA7-0F056AD99E91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA084F11-C5BC-4FA6-9AE3-D8BE91A1D8C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23550" yWindow="-1290" windowWidth="20205" windowHeight="13395" xr2:uid="{711B29A3-FC20-40C1-A5E5-A5DE4D99F3B8}"/>
+    <workbookView xWindow="4452" yWindow="1212" windowWidth="14700" windowHeight="10236" xr2:uid="{711B29A3-FC20-40C1-A5E5-A5DE4D99F3B8}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,18 +36,75 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
-  <si>
-    <t>Equation Num</t>
-  </si>
-  <si>
-    <t>Equation Desc</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
   <si>
     <t>Function</t>
   </si>
   <si>
     <t>File</t>
+  </si>
+  <si>
+    <t>Eq_Code</t>
+  </si>
+  <si>
+    <t>Ex_Num</t>
+  </si>
+  <si>
+    <t>Eq_Desc</t>
+  </si>
+  <si>
+    <t>SpawnOutput</t>
+  </si>
+  <si>
+    <t>EggSmoltBH</t>
+  </si>
+  <si>
+    <t>SmoltProdRicker</t>
+  </si>
+  <si>
+    <t>EggProdHabitat</t>
+  </si>
+  <si>
+    <t>FryProdHabitat</t>
+  </si>
+  <si>
+    <t>SmoltProdHabitat</t>
+  </si>
+  <si>
+    <t>HockeyStick</t>
+  </si>
+  <si>
+    <t>Broodtake</t>
+  </si>
+  <si>
+    <t>BroodtakeImportStray</t>
+  </si>
+  <si>
+    <t>EggProd</t>
+  </si>
+  <si>
+    <t>EggTarget</t>
+  </si>
+  <si>
+    <t>pBroodtake</t>
+  </si>
+  <si>
+    <t>ProdYearSubYear</t>
+  </si>
+  <si>
+    <t>SmoltRel1</t>
+  </si>
+  <si>
+    <t>SmoltRel2</t>
+  </si>
+  <si>
+    <t>Eggsum</t>
+  </si>
+  <si>
+    <t>YearlingTarget</t>
+  </si>
+  <si>
+    <t>SubyearlingTarget</t>
   </si>
 </sst>
 </file>
@@ -419,47 +476,121 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73880E9D-B707-44BB-BDFC-1893328C0FC3}">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.5546875" customWidth="1"/>
-    <col min="2" max="2" width="15.109375" customWidth="1"/>
-    <col min="3" max="3" width="11.109375" customWidth="1"/>
-    <col min="4" max="4" width="10.109375" customWidth="1"/>
+    <col min="1" max="1" width="18.33203125" customWidth="1"/>
+    <col min="2" max="2" width="17.5546875" customWidth="1"/>
+    <col min="3" max="3" width="22.44140625" customWidth="1"/>
+    <col min="4" max="4" width="11.109375" customWidth="1"/>
+    <col min="5" max="5" width="10.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="E1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5">
-        <v>4</v>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>